<commit_message>
fix: restore all lost files after filter-branch
</commit_message>
<xml_diff>
--- a/public/templates/mau_nhap_du_lieu.xlsx
+++ b/public/templates/mau_nhap_du_lieu.xlsx
@@ -27,14 +27,20 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,7 +57,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,24 +428,24 @@
   <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,7 +506,7 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Tên nhà thầu</t>
+          <t>Tên nhà thầu (Bên B)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">

</xml_diff>